<commit_message>
added the info for swedish archetypes and the cost factors for the design of the cables
</commit_message>
<xml_diff>
--- a/eureca_ubem/Input/materials_uppsala_sodermans.xlsx
+++ b/eureca_ubem/Input/materials_uppsala_sodermans.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Works\EUReCA\EUReCA\eureca_ubem\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5348364A-2981-4160-AEA3-697452BB5BA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F518ED4-651E-4C74-80B8-2E56A93D2785}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="823" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4152" yWindow="2244" windowWidth="17280" windowHeight="8880" tabRatio="823" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Envelopes" sheetId="2" r:id="rId1"/>
@@ -121,7 +121,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="75">
   <si>
     <t>id</t>
   </si>
@@ -263,6 +263,90 @@
   <si>
     <t>Medium</t>
   </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
+    <t>D+</t>
+  </si>
+  <si>
+    <t>C+</t>
+  </si>
+  <si>
+    <t>B+</t>
+  </si>
+  <si>
+    <t>A+</t>
+  </si>
+  <si>
+    <t>E+</t>
+  </si>
+  <si>
+    <t>D++</t>
+  </si>
+  <si>
+    <t>C++</t>
+  </si>
+  <si>
+    <t>B++</t>
+  </si>
+  <si>
+    <t>A++</t>
+  </si>
+  <si>
+    <t>E++</t>
+  </si>
+  <si>
+    <t>D+++</t>
+  </si>
+  <si>
+    <t>C+++</t>
+  </si>
+  <si>
+    <t>B+++</t>
+  </si>
+  <si>
+    <t>A+++</t>
+  </si>
+  <si>
+    <t>E+++</t>
+  </si>
+  <si>
+    <t>SFH_before_1960</t>
+  </si>
+  <si>
+    <t>SFH_1961_1975</t>
+  </si>
+  <si>
+    <t>SFH_1976_1985</t>
+  </si>
+  <si>
+    <t>SFH_1986_1995</t>
+  </si>
+  <si>
+    <t>SFH_1996_2005</t>
+  </si>
+  <si>
+    <t>SFH_after_2006</t>
+  </si>
+  <si>
+    <t>MFH_before_1960</t>
+  </si>
+  <si>
+    <t>MFH_1961_1975</t>
+  </si>
+  <si>
+    <t>MFH_1976_1985</t>
+  </si>
+  <si>
+    <t>MFH_1986_1995</t>
+  </si>
+  <si>
+    <t>MFH_1996_2005</t>
+  </si>
+  <si>
+    <t>MFH_after_2006</t>
+  </si>
 </sst>
 </file>
 
@@ -271,7 +355,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -322,6 +406,12 @@
       <color indexed="81"/>
       <name val="Tahoma"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -830,11 +920,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:AMJ19"/>
+  <dimension ref="A1:AMJ69"/>
   <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.33203125" style="7" customWidth="1"/>
-    <col min="2" max="4" width="12.6640625" style="7" customWidth="1"/>
+    <col min="2" max="2" width="18.33203125" style="7" customWidth="1"/>
+    <col min="3" max="4" width="12.6640625" style="7" customWidth="1"/>
     <col min="5" max="5" width="12.5546875" style="7" customWidth="1"/>
     <col min="6" max="6" width="13.5546875" style="7" customWidth="1"/>
     <col min="7" max="7" width="10.88671875" style="7" customWidth="1"/>
@@ -883,26 +974,8 @@
       <c r="A2" s="7">
         <v>1</v>
       </c>
-      <c r="B2" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="C2" s="8">
-        <v>11</v>
-      </c>
-      <c r="D2" s="8">
-        <v>12</v>
-      </c>
-      <c r="E2" s="8">
-        <v>13</v>
-      </c>
-      <c r="F2" s="8">
-        <v>14</v>
-      </c>
-      <c r="G2" s="8">
-        <v>15</v>
-      </c>
-      <c r="H2" s="8">
-        <v>16</v>
+      <c r="B2" s="6" t="s">
+        <v>63</v>
       </c>
       <c r="AMA2" s="7"/>
       <c r="AMB2" s="7"/>
@@ -919,26 +992,8 @@
       <c r="A3" s="7">
         <v>2</v>
       </c>
-      <c r="B3" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="C3" s="8">
-        <v>31</v>
-      </c>
-      <c r="D3" s="8">
-        <v>32</v>
-      </c>
-      <c r="E3" s="8">
-        <v>33</v>
-      </c>
-      <c r="F3" s="8">
-        <v>34</v>
-      </c>
-      <c r="G3" s="8">
-        <v>35</v>
-      </c>
-      <c r="H3" s="8">
-        <v>36</v>
+      <c r="B3" s="6" t="s">
+        <v>64</v>
       </c>
       <c r="AMA3" s="7"/>
       <c r="AMB3" s="7"/>
@@ -955,26 +1010,8 @@
       <c r="A4" s="7">
         <v>3</v>
       </c>
-      <c r="B4" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="C4" s="8">
-        <v>41</v>
-      </c>
-      <c r="D4" s="8">
-        <v>42</v>
-      </c>
-      <c r="E4" s="8">
-        <v>43</v>
-      </c>
-      <c r="F4" s="8">
-        <v>44</v>
-      </c>
-      <c r="G4" s="8">
-        <v>45</v>
-      </c>
-      <c r="H4" s="8">
-        <v>46</v>
+      <c r="B4" s="6" t="s">
+        <v>65</v>
       </c>
       <c r="AMA4" s="7"/>
       <c r="AMB4" s="7"/>
@@ -992,25 +1029,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="C5" s="8">
-        <v>51</v>
-      </c>
-      <c r="D5" s="8">
-        <v>52</v>
-      </c>
-      <c r="E5" s="8">
-        <v>53</v>
-      </c>
-      <c r="F5" s="8">
-        <v>54</v>
-      </c>
-      <c r="G5" s="8">
-        <v>55</v>
-      </c>
-      <c r="H5" s="8">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="AMA5" s="7"/>
       <c r="AMB5" s="7"/>
@@ -1024,14 +1043,12 @@
       <c r="AMJ5" s="7"/>
     </row>
     <row r="6" spans="1:1024" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="7"/>
-      <c r="B6" s="7"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="8"/>
-      <c r="H6" s="8"/>
+      <c r="A6" s="7">
+        <v>5</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>67</v>
+      </c>
       <c r="AMA6" s="7"/>
       <c r="AMB6" s="7"/>
       <c r="AMC6" s="7"/>
@@ -1044,14 +1061,12 @@
       <c r="AMJ6" s="7"/>
     </row>
     <row r="7" spans="1:1024" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="7"/>
-      <c r="B7" s="7"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="8"/>
+      <c r="A7" s="7">
+        <v>6</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>68</v>
+      </c>
       <c r="AMA7" s="7"/>
       <c r="AMB7" s="7"/>
       <c r="AMC7" s="7"/>
@@ -1064,14 +1079,12 @@
       <c r="AMJ7" s="7"/>
     </row>
     <row r="8" spans="1:1024" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="7"/>
-      <c r="B8" s="7"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="8"/>
+      <c r="A8" s="7">
+        <v>7</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>69</v>
+      </c>
       <c r="AMA8" s="7"/>
       <c r="AMB8" s="7"/>
       <c r="AMC8" s="7"/>
@@ -1084,14 +1097,12 @@
       <c r="AMJ8" s="7"/>
     </row>
     <row r="9" spans="1:1024" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="7"/>
-      <c r="B9" s="7"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="8"/>
+      <c r="A9" s="7">
+        <v>8</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>70</v>
+      </c>
       <c r="AMA9" s="7"/>
       <c r="AMB9" s="7"/>
       <c r="AMC9" s="7"/>
@@ -1104,14 +1115,12 @@
       <c r="AMJ9" s="7"/>
     </row>
     <row r="10" spans="1:1024" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="7"/>
-      <c r="B10" s="7"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
-      <c r="H10" s="8"/>
+      <c r="A10" s="7">
+        <v>9</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>71</v>
+      </c>
       <c r="AMA10" s="7"/>
       <c r="AMB10" s="7"/>
       <c r="AMC10" s="7"/>
@@ -1124,6 +1133,12 @@
       <c r="AMJ10" s="7"/>
     </row>
     <row r="11" spans="1:1024" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="7">
+        <v>10</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>72</v>
+      </c>
       <c r="ALZ11" s="7"/>
       <c r="AMA11" s="7"/>
       <c r="AMB11" s="7"/>
@@ -1136,6 +1151,12 @@
       <c r="AMI11" s="7"/>
     </row>
     <row r="12" spans="1:1024" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="7">
+        <v>11</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>73</v>
+      </c>
       <c r="ALZ12" s="7"/>
       <c r="AMA12" s="7"/>
       <c r="AMB12" s="7"/>
@@ -1148,6 +1169,12 @@
       <c r="AMI12" s="7"/>
     </row>
     <row r="13" spans="1:1024" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="7">
+        <v>12</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>74</v>
+      </c>
       <c r="ALZ13" s="7"/>
       <c r="AMA13" s="7"/>
       <c r="AMB13" s="7"/>
@@ -1160,36 +1187,815 @@
       <c r="AMI13" s="7"/>
     </row>
     <row r="14" spans="1:1024" x14ac:dyDescent="0.3">
-      <c r="A14" s="6"/>
-      <c r="B14" s="6"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6"/>
-      <c r="G14" s="6"/>
+      <c r="A14" s="7">
+        <v>13</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="15" spans="1:1024" x14ac:dyDescent="0.3">
-      <c r="A15" s="6"/>
-      <c r="B15" s="6"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
+      <c r="A15" s="7">
+        <v>14</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="16" spans="1:1024" x14ac:dyDescent="0.3">
-      <c r="A16" s="6"/>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A17" s="6"/>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A18" s="6"/>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A19" s="6"/>
+      <c r="A16" s="7">
+        <v>15</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" s="7">
+        <v>16</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" s="7">
+        <v>17</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" s="7">
+        <v>18</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" s="7">
+        <v>19</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" s="7">
+        <v>20</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22" s="7">
+        <v>21</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A23" s="7">
+        <v>22</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A24" s="7">
+        <v>23</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A25" s="7">
+        <v>24</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A26" s="7">
+        <v>25</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A27" s="7">
+        <v>26</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A28" s="7">
+        <v>27</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A29" s="7">
+        <v>28</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A30" s="7">
+        <v>29</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A31" s="7">
+        <v>30</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A32" s="7">
+        <v>31</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A33" s="7">
+        <v>32</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A34" s="7">
+        <v>33</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A35" s="7">
+        <v>34</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A36" s="7">
+        <v>35</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A37" s="7">
+        <v>36</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A38" s="7">
+        <v>37</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A39" s="7">
+        <v>38</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A40" s="7">
+        <v>39</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A41" s="7">
+        <v>40</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A42" s="7">
+        <v>41</v>
+      </c>
+      <c r="B42" s="6" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A43" s="7">
+        <v>42</v>
+      </c>
+      <c r="B43" s="6" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A44" s="7">
+        <v>43</v>
+      </c>
+      <c r="B44" s="6" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A45" s="7">
+        <v>44</v>
+      </c>
+      <c r="B45" s="6" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A46" s="7">
+        <v>45</v>
+      </c>
+      <c r="B46" s="6" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A47" s="7">
+        <v>46</v>
+      </c>
+      <c r="B47" s="6" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A48" s="7">
+        <v>47</v>
+      </c>
+      <c r="B48" s="6" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A49" s="7">
+        <v>48</v>
+      </c>
+      <c r="B49" s="6" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A50" s="7">
+        <v>49</v>
+      </c>
+      <c r="B50" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="C50" s="8">
+        <v>11</v>
+      </c>
+      <c r="D50" s="8">
+        <v>12</v>
+      </c>
+      <c r="E50" s="8">
+        <v>13</v>
+      </c>
+      <c r="F50" s="8">
+        <v>14</v>
+      </c>
+      <c r="G50" s="8">
+        <v>15</v>
+      </c>
+      <c r="H50" s="8">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A51" s="7">
+        <v>50</v>
+      </c>
+      <c r="B51" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C51" s="8">
+        <v>31</v>
+      </c>
+      <c r="D51" s="8">
+        <v>32</v>
+      </c>
+      <c r="E51" s="8">
+        <v>33</v>
+      </c>
+      <c r="F51" s="8">
+        <v>34</v>
+      </c>
+      <c r="G51" s="8">
+        <v>35</v>
+      </c>
+      <c r="H51" s="8">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A52" s="7">
+        <v>51</v>
+      </c>
+      <c r="B52" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C52" s="8">
+        <v>41</v>
+      </c>
+      <c r="D52" s="8">
+        <v>42</v>
+      </c>
+      <c r="E52" s="8">
+        <v>43</v>
+      </c>
+      <c r="F52" s="8">
+        <v>44</v>
+      </c>
+      <c r="G52" s="8">
+        <v>45</v>
+      </c>
+      <c r="H52" s="8">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A53" s="7">
+        <v>52</v>
+      </c>
+      <c r="B53" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C53" s="8">
+        <v>51</v>
+      </c>
+      <c r="D53" s="8">
+        <v>52</v>
+      </c>
+      <c r="E53" s="8">
+        <v>53</v>
+      </c>
+      <c r="F53" s="8">
+        <v>54</v>
+      </c>
+      <c r="G53" s="8">
+        <v>55</v>
+      </c>
+      <c r="H53" s="8">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A54" s="7">
+        <v>53</v>
+      </c>
+      <c r="B54" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="C54" s="8">
+        <v>51</v>
+      </c>
+      <c r="D54" s="8">
+        <v>52</v>
+      </c>
+      <c r="E54" s="8">
+        <v>53</v>
+      </c>
+      <c r="F54" s="8">
+        <v>54</v>
+      </c>
+      <c r="G54" s="8">
+        <v>55</v>
+      </c>
+      <c r="H54" s="8">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A55" s="7">
+        <v>54</v>
+      </c>
+      <c r="B55" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="C55" s="8">
+        <v>11</v>
+      </c>
+      <c r="D55" s="8">
+        <v>12</v>
+      </c>
+      <c r="E55" s="8">
+        <v>13</v>
+      </c>
+      <c r="F55" s="8">
+        <v>14</v>
+      </c>
+      <c r="G55" s="8">
+        <v>15</v>
+      </c>
+      <c r="H55" s="8">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A56" s="7">
+        <v>55</v>
+      </c>
+      <c r="B56" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C56" s="8">
+        <v>31</v>
+      </c>
+      <c r="D56" s="8">
+        <v>32</v>
+      </c>
+      <c r="E56" s="8">
+        <v>33</v>
+      </c>
+      <c r="F56" s="8">
+        <v>34</v>
+      </c>
+      <c r="G56" s="8">
+        <v>35</v>
+      </c>
+      <c r="H56" s="8">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A57" s="7">
+        <v>56</v>
+      </c>
+      <c r="B57" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="C57" s="8">
+        <v>41</v>
+      </c>
+      <c r="D57" s="8">
+        <v>42</v>
+      </c>
+      <c r="E57" s="8">
+        <v>43</v>
+      </c>
+      <c r="F57" s="8">
+        <v>44</v>
+      </c>
+      <c r="G57" s="8">
+        <v>45</v>
+      </c>
+      <c r="H57" s="8">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A58" s="7">
+        <v>57</v>
+      </c>
+      <c r="B58" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C58" s="8">
+        <v>51</v>
+      </c>
+      <c r="D58" s="8">
+        <v>52</v>
+      </c>
+      <c r="E58" s="8">
+        <v>53</v>
+      </c>
+      <c r="F58" s="8">
+        <v>54</v>
+      </c>
+      <c r="G58" s="8">
+        <v>55</v>
+      </c>
+      <c r="H58" s="8">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A59" s="7">
+        <v>58</v>
+      </c>
+      <c r="B59" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C59" s="8">
+        <v>51</v>
+      </c>
+      <c r="D59" s="8">
+        <v>52</v>
+      </c>
+      <c r="E59" s="8">
+        <v>53</v>
+      </c>
+      <c r="F59" s="8">
+        <v>54</v>
+      </c>
+      <c r="G59" s="8">
+        <v>55</v>
+      </c>
+      <c r="H59" s="8">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A60" s="7">
+        <v>59</v>
+      </c>
+      <c r="B60" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="C60" s="8">
+        <v>11</v>
+      </c>
+      <c r="D60" s="8">
+        <v>12</v>
+      </c>
+      <c r="E60" s="8">
+        <v>13</v>
+      </c>
+      <c r="F60" s="8">
+        <v>14</v>
+      </c>
+      <c r="G60" s="8">
+        <v>15</v>
+      </c>
+      <c r="H60" s="8">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A61" s="7">
+        <v>60</v>
+      </c>
+      <c r="B61" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="C61" s="8">
+        <v>31</v>
+      </c>
+      <c r="D61" s="8">
+        <v>32</v>
+      </c>
+      <c r="E61" s="8">
+        <v>33</v>
+      </c>
+      <c r="F61" s="8">
+        <v>34</v>
+      </c>
+      <c r="G61" s="8">
+        <v>35</v>
+      </c>
+      <c r="H61" s="8">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A62" s="7">
+        <v>61</v>
+      </c>
+      <c r="B62" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="C62" s="8">
+        <v>41</v>
+      </c>
+      <c r="D62" s="8">
+        <v>42</v>
+      </c>
+      <c r="E62" s="8">
+        <v>43</v>
+      </c>
+      <c r="F62" s="8">
+        <v>44</v>
+      </c>
+      <c r="G62" s="8">
+        <v>45</v>
+      </c>
+      <c r="H62" s="8">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A63" s="7">
+        <v>62</v>
+      </c>
+      <c r="B63" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="C63" s="8">
+        <v>51</v>
+      </c>
+      <c r="D63" s="8">
+        <v>52</v>
+      </c>
+      <c r="E63" s="8">
+        <v>53</v>
+      </c>
+      <c r="F63" s="8">
+        <v>54</v>
+      </c>
+      <c r="G63" s="8">
+        <v>55</v>
+      </c>
+      <c r="H63" s="8">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A64" s="7">
+        <v>63</v>
+      </c>
+      <c r="B64" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="C64" s="8">
+        <v>51</v>
+      </c>
+      <c r="D64" s="8">
+        <v>52</v>
+      </c>
+      <c r="E64" s="8">
+        <v>53</v>
+      </c>
+      <c r="F64" s="8">
+        <v>54</v>
+      </c>
+      <c r="G64" s="8">
+        <v>55</v>
+      </c>
+      <c r="H64" s="8">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A65" s="7">
+        <v>64</v>
+      </c>
+      <c r="B65" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="C65" s="8">
+        <v>11</v>
+      </c>
+      <c r="D65" s="8">
+        <v>12</v>
+      </c>
+      <c r="E65" s="8">
+        <v>13</v>
+      </c>
+      <c r="F65" s="8">
+        <v>14</v>
+      </c>
+      <c r="G65" s="8">
+        <v>15</v>
+      </c>
+      <c r="H65" s="8">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A66" s="7">
+        <v>65</v>
+      </c>
+      <c r="B66" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="C66" s="8">
+        <v>31</v>
+      </c>
+      <c r="D66" s="8">
+        <v>32</v>
+      </c>
+      <c r="E66" s="8">
+        <v>33</v>
+      </c>
+      <c r="F66" s="8">
+        <v>34</v>
+      </c>
+      <c r="G66" s="8">
+        <v>35</v>
+      </c>
+      <c r="H66" s="8">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A67" s="7">
+        <v>66</v>
+      </c>
+      <c r="B67" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="C67" s="8">
+        <v>41</v>
+      </c>
+      <c r="D67" s="8">
+        <v>42</v>
+      </c>
+      <c r="E67" s="8">
+        <v>43</v>
+      </c>
+      <c r="F67" s="8">
+        <v>44</v>
+      </c>
+      <c r="G67" s="8">
+        <v>45</v>
+      </c>
+      <c r="H67" s="8">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A68" s="7">
+        <v>67</v>
+      </c>
+      <c r="B68" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="C68" s="8">
+        <v>51</v>
+      </c>
+      <c r="D68" s="8">
+        <v>52</v>
+      </c>
+      <c r="E68" s="8">
+        <v>53</v>
+      </c>
+      <c r="F68" s="8">
+        <v>54</v>
+      </c>
+      <c r="G68" s="8">
+        <v>55</v>
+      </c>
+      <c r="H68" s="8">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A69" s="7">
+        <v>68</v>
+      </c>
+      <c r="B69" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="C69" s="8">
+        <v>51</v>
+      </c>
+      <c r="D69" s="8">
+        <v>52</v>
+      </c>
+      <c r="E69" s="8">
+        <v>53</v>
+      </c>
+      <c r="F69" s="8">
+        <v>54</v>
+      </c>
+      <c r="G69" s="8">
+        <v>55</v>
+      </c>
+      <c r="H69" s="8">
+        <v>56</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="8" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
@@ -8864,6 +9670,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100B4A72D35825A314C9EB5C5BDD49EC582" ma:contentTypeVersion="10" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="ab3cfd4ffe88710ffd03436b1addd592">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="c0574b82-72ca-428d-96cb-9dbc44012ede" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fb55e547d0e393e34c6bbb534eb78df0" ns3:_="">
     <xsd:import namespace="c0574b82-72ca-428d-96cb-9dbc44012ede"/>
@@ -9047,15 +9862,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
@@ -9063,6 +9869,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D8F108CF-CFD9-47FB-AD65-C74A1CC8D454}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D81EF3F0-7775-4285-BFE0-18A3A29E794A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9076,14 +9890,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D8F108CF-CFD9-47FB-AD65-C74A1CC8D454}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>